<commit_message>
Makni reference na GOS sa stranice i iz Excel tablica
- Podnožje: bez GOS kontakta i izvora; ostaje link na Excel raspored.
- Napomene o biootpadu i kraju rasporeda bez spominjanja GOS-a.
- Excel: bez retka s izvorom i GOS kontakta u napomenama.
- Meta opis stranice bez GOS-a; uklonjeno nekorišteno polje "src" iz podataka.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012grr9UJafq4ZimrFiB6wUv
</commit_message>
<xml_diff>
--- a/excel/Raspored_odvoza_Zona10_2026.xlsx
+++ b/excel/Raspored_odvoza_Zona10_2026.xlsx
@@ -1116,7 +1116,7 @@
     <row r="30">
       <c r="A30" s="21" t="inlineStr">
         <is>
-          <t>• Spremnike iznijeti na javnu površinu najkasnije do 07:00. Info: 0800 200 214, info@gos.hr, www.gos.hr</t>
+          <t>• Spremnike iznijeti na javnu površinu najkasnije do 07:00.</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Izvor: GOS d.o.o., RASPORED_2026_Zona_10.pdf. "x" = odvoz tog dana. Spremnike iznijeti do 07:00. Prošli datumi su posivljeni.</t>
+          <t>"x" = odvoz tog dana. Spremnike iznijeti do 07:00. Prošli datumi su posivljeni.</t>
         </is>
       </c>
     </row>

</xml_diff>